<commit_message>
Update CORE-000580 rule tests
</commit_message>
<xml_diff>
--- a/rules/CORE-000580/positive/02/data/unit-test-coreid-CG0325-positive02.xlsx
+++ b/rules/CORE-000580/positive/02/data/unit-test-coreid-CG0325-positive02.xlsx
@@ -1,23 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\verisian\core-contributor\rules\CORE-000580\positive\02\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{820298B5-3D71-45FB-ADBF-D17D24E75FD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46EEEDB5-B9D7-4F0D-BE17-E9A4B9AD2470}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11265" yWindow="435" windowWidth="15450" windowHeight="14505" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
     <sheet name="Datasets" sheetId="2" r:id="rId2"/>
     <sheet name="te.xpt" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -247,7 +260,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -604,6 +617,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:I12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="5" max="5" width="21" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
@@ -697,7 +713,7 @@
       <c r="H4" s="6"/>
       <c r="I4" s="6"/>
     </row>
-    <row r="5" spans="1:9" ht="120" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>21</v>
       </c>
@@ -715,7 +731,7 @@
       </c>
       <c r="F5" s="5"/>
     </row>
-    <row r="6" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>21</v>
       </c>
@@ -735,7 +751,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>21</v>
       </c>
@@ -755,7 +771,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="120" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>21</v>
       </c>
@@ -773,7 +789,7 @@
       </c>
       <c r="F8" s="5"/>
     </row>
-    <row r="9" spans="1:9" ht="120" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>21</v>
       </c>
@@ -791,7 +807,7 @@
       </c>
       <c r="F9" s="5"/>
     </row>
-    <row r="10" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>21</v>
       </c>
@@ -809,7 +825,7 @@
       </c>
       <c r="F10" s="5"/>
     </row>
-    <row r="11" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>21</v>
       </c>
@@ -827,7 +843,7 @@
       </c>
       <c r="F11" s="5"/>
     </row>
-    <row r="12" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>21</v>
       </c>

</xml_diff>